<commit_message>
minor changes in week 2
</commit_message>
<xml_diff>
--- a/Week_02 - Hello, Machine Learning/Data Science/model_report.xlsx
+++ b/Week_02 - Hello, Machine Learning/Data Science/model_report.xlsx
@@ -16,7 +16,6 @@
     <sheet name="KNN_hyperparameter_tuning" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -41,7 +40,7 @@
     <t>Comment</t>
   </si>
   <si>
-    <t>We see that leaf_size does not play a role in the accuracy. P=1 and p=3 both decrease it. The best models are the ones with 5 neighboors and p=2</t>
+    <t>leaf_size doesn't seem to affect the performance of the model. P=1 and p=0 make the accuracy worse. The best models are those with k=5 and p=2</t>
   </si>
 </sst>
 </file>
@@ -71,7 +70,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -214,26 +213,42 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -566,8 +581,7 @@
   <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.42578125" customWidth="1"/>
-    <col min="3" max="3" width="13.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -853,14 +867,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J109"/>
+  <dimension ref="A1:I109"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="13.42578125" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="4" max="4" width="11.28515625" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -876,13 +890,13 @@
       <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="5"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -898,13 +912,13 @@
       <c r="E2">
         <v>0.86</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="2"/>
-      <c r="J2" s="7"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H2" s="4"/>
+      <c r="I2" s="5"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -920,11 +934,11 @@
       <c r="E3">
         <v>0.84599999999999997</v>
       </c>
-      <c r="H3" s="6"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="7"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G3" s="6"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="8"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -940,11 +954,11 @@
       <c r="E4">
         <v>0.84299999999999997</v>
       </c>
-      <c r="H4" s="6"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="7"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G4" s="6"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="8"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -960,11 +974,11 @@
       <c r="E5">
         <v>0.86</v>
       </c>
-      <c r="H5" s="6"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="7"/>
-    </row>
-    <row r="6" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G5" s="6"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="8"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
@@ -980,11 +994,11 @@
       <c r="E6">
         <v>0.84599999999999997</v>
       </c>
-      <c r="H6" s="8"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="10"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G6" s="6"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="8"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
@@ -1000,8 +1014,11 @@
       <c r="E7">
         <v>0.84299999999999997</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G7" s="6"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="8"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1</v>
       </c>
@@ -1017,8 +1034,11 @@
       <c r="E8">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G8" s="6"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="8"/>
+    </row>
+    <row r="9" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1</v>
       </c>
@@ -1034,8 +1054,11 @@
       <c r="E9">
         <v>0.84599999999999997</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G9" s="9"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="11"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1</v>
       </c>
@@ -1052,7 +1075,7 @@
         <v>0.84299999999999997</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1</v>
       </c>
@@ -1069,7 +1092,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>1</v>
       </c>
@@ -1086,7 +1109,7 @@
         <v>0.84599999999999997</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1</v>
       </c>
@@ -1103,7 +1126,7 @@
         <v>0.84299999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2</v>
       </c>
@@ -1120,7 +1143,7 @@
         <v>0.876</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2</v>
       </c>
@@ -1137,7 +1160,7 @@
         <v>0.872</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2</v>
       </c>
@@ -2737,8 +2760,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="H2:J6"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="G2:I9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>